<commit_message>
Suggestions Implemented - 1
</commit_message>
<xml_diff>
--- a/Task-1/mock_data/client_summary.xlsx
+++ b/Task-1/mock_data/client_summary.xlsx
@@ -485,13 +485,13 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>65000</v>
+        <v>64086</v>
       </c>
       <c r="G2" t="n">
-        <v>9750</v>
+        <v>9612</v>
       </c>
       <c r="H2" t="n">
-        <v>55250</v>
+        <v>54474</v>
       </c>
     </row>
     <row r="3">
@@ -521,13 +521,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>65000</v>
+        <v>66015</v>
       </c>
       <c r="G3" t="n">
-        <v>9750</v>
+        <v>9902</v>
       </c>
       <c r="H3" t="n">
-        <v>55250</v>
+        <v>56113</v>
       </c>
     </row>
     <row r="4">
@@ -557,13 +557,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>65000</v>
+        <v>74997</v>
       </c>
       <c r="G4" t="n">
-        <v>9750</v>
+        <v>11249</v>
       </c>
       <c r="H4" t="n">
-        <v>55250</v>
+        <v>63748</v>
       </c>
     </row>
     <row r="5">
@@ -584,22 +584,22 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2019-05-01</t>
+          <t>2019-04-01</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>May 2019</t>
+          <t>Apr 2019</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>65000</v>
+        <v>65010</v>
       </c>
       <c r="G5" t="n">
-        <v>9750</v>
+        <v>9751</v>
       </c>
       <c r="H5" t="n">
-        <v>55250</v>
+        <v>55259</v>
       </c>
     </row>
     <row r="6">
@@ -620,22 +620,22 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2019-06-01</t>
+          <t>2019-05-01</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Jun 2019</t>
+          <t>May 2019</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>65000</v>
+        <v>63932</v>
       </c>
       <c r="G6" t="n">
-        <v>9750</v>
+        <v>9589</v>
       </c>
       <c r="H6" t="n">
-        <v>55250</v>
+        <v>54343</v>
       </c>
     </row>
     <row r="7">
@@ -656,22 +656,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2019-07-01</t>
+          <t>2019-06-01</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Jul 2019</t>
+          <t>Jun 2019</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>65000</v>
+        <v>79033</v>
       </c>
       <c r="G7" t="n">
-        <v>9750</v>
+        <v>11854</v>
       </c>
       <c r="H7" t="n">
-        <v>55250</v>
+        <v>67179</v>
       </c>
     </row>
     <row r="8">
@@ -692,22 +692,22 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2019-08-01</t>
+          <t>2019-07-01</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Aug 2019</t>
+          <t>Jul 2019</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>65000</v>
+        <v>63903</v>
       </c>
       <c r="G8" t="n">
-        <v>9750</v>
+        <v>9585</v>
       </c>
       <c r="H8" t="n">
-        <v>55250</v>
+        <v>54318</v>
       </c>
     </row>
     <row r="9">
@@ -728,22 +728,22 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2019-10-01</t>
+          <t>2019-08-01</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Oct 2019</t>
+          <t>Aug 2019</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>65000</v>
+        <v>63797</v>
       </c>
       <c r="G9" t="n">
-        <v>9750</v>
+        <v>9569</v>
       </c>
       <c r="H9" t="n">
-        <v>55250</v>
+        <v>54228</v>
       </c>
     </row>
     <row r="10">
@@ -764,22 +764,22 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2019-11-01</t>
+          <t>2019-09-01</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Nov 2019</t>
+          <t>Sep 2019</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>65000</v>
+        <v>81057</v>
       </c>
       <c r="G10" t="n">
-        <v>9750</v>
+        <v>12158</v>
       </c>
       <c r="H10" t="n">
-        <v>55250</v>
+        <v>68899</v>
       </c>
     </row>
     <row r="11">
@@ -800,22 +800,22 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2019-12-01</t>
+          <t>2019-10-01</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Dec 2019</t>
+          <t>Oct 2019</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>65000</v>
+        <v>66271</v>
       </c>
       <c r="G11" t="n">
-        <v>9750</v>
+        <v>9940</v>
       </c>
       <c r="H11" t="n">
-        <v>55250</v>
+        <v>56331</v>
       </c>
     </row>
     <row r="12">
@@ -836,22 +836,22 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2020-01-01</t>
+          <t>2019-11-01</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Jan 2020</t>
+          <t>Nov 2019</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>68250</v>
+        <v>64630</v>
       </c>
       <c r="G12" t="n">
-        <v>10237</v>
+        <v>9694</v>
       </c>
       <c r="H12" t="n">
-        <v>58013</v>
+        <v>54936</v>
       </c>
     </row>
     <row r="13">
@@ -872,22 +872,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2020-02-01</t>
+          <t>2019-12-01</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Feb 2020</t>
+          <t>Dec 2019</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>68250</v>
+        <v>108635</v>
       </c>
       <c r="G13" t="n">
-        <v>10237</v>
+        <v>16295</v>
       </c>
       <c r="H13" t="n">
-        <v>58013</v>
+        <v>92340</v>
       </c>
     </row>
     <row r="14">
@@ -908,22 +908,22 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2020-03-01</t>
+          <t>2020-01-01</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Mar 2020</t>
+          <t>Jan 2020</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>68250</v>
+        <v>65537</v>
       </c>
       <c r="G14" t="n">
-        <v>10237</v>
+        <v>9830</v>
       </c>
       <c r="H14" t="n">
-        <v>58013</v>
+        <v>55707</v>
       </c>
     </row>
     <row r="15">
@@ -944,22 +944,22 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2020-04-01</t>
+          <t>2020-03-01</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Apr 2020</t>
+          <t>Mar 2020</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>68250</v>
+        <v>77991</v>
       </c>
       <c r="G15" t="n">
-        <v>10237</v>
+        <v>11698</v>
       </c>
       <c r="H15" t="n">
-        <v>58013</v>
+        <v>66293</v>
       </c>
     </row>
     <row r="16">
@@ -980,22 +980,22 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2020-05-01</t>
+          <t>2020-04-01</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>May 2020</t>
+          <t>Apr 2020</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>68250</v>
+        <v>64824</v>
       </c>
       <c r="G16" t="n">
-        <v>10237</v>
+        <v>9723</v>
       </c>
       <c r="H16" t="n">
-        <v>58013</v>
+        <v>55101</v>
       </c>
     </row>
     <row r="17">
@@ -1016,22 +1016,22 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2020-07-01</t>
+          <t>2020-05-01</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Jul 2020</t>
+          <t>May 2020</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>68250</v>
+        <v>63875</v>
       </c>
       <c r="G17" t="n">
-        <v>10237</v>
+        <v>9581</v>
       </c>
       <c r="H17" t="n">
-        <v>58013</v>
+        <v>54294</v>
       </c>
     </row>
     <row r="18">
@@ -1052,22 +1052,22 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2020-08-01</t>
+          <t>2020-07-01</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Aug 2020</t>
+          <t>Jul 2020</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>68250</v>
+        <v>65736</v>
       </c>
       <c r="G18" t="n">
-        <v>10237</v>
+        <v>9860</v>
       </c>
       <c r="H18" t="n">
-        <v>58013</v>
+        <v>55876</v>
       </c>
     </row>
     <row r="19">
@@ -1088,22 +1088,22 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2020-09-01</t>
+          <t>2020-08-01</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Sep 2020</t>
+          <t>Aug 2020</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>68250</v>
+        <v>64635</v>
       </c>
       <c r="G19" t="n">
-        <v>10237</v>
+        <v>9695</v>
       </c>
       <c r="H19" t="n">
-        <v>58013</v>
+        <v>54940</v>
       </c>
     </row>
     <row r="20">
@@ -1124,22 +1124,22 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2020-10-01</t>
+          <t>2020-09-01</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Oct 2020</t>
+          <t>Sep 2020</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>68250</v>
+        <v>82356</v>
       </c>
       <c r="G20" t="n">
-        <v>10237</v>
+        <v>12353</v>
       </c>
       <c r="H20" t="n">
-        <v>58013</v>
+        <v>70003</v>
       </c>
     </row>
     <row r="21">
@@ -1160,22 +1160,22 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2020-11-01</t>
+          <t>2020-10-01</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Nov 2020</t>
+          <t>Oct 2020</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>68250</v>
+        <v>64837</v>
       </c>
       <c r="G21" t="n">
-        <v>10237</v>
+        <v>9725</v>
       </c>
       <c r="H21" t="n">
-        <v>58013</v>
+        <v>55112</v>
       </c>
     </row>
     <row r="22">
@@ -1205,13 +1205,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>68250</v>
+        <v>124239</v>
       </c>
       <c r="G22" t="n">
-        <v>10237</v>
+        <v>18635</v>
       </c>
       <c r="H22" t="n">
-        <v>58013</v>
+        <v>105604</v>
       </c>
     </row>
     <row r="23">
@@ -1241,13 +1241,13 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>71662</v>
+        <v>64483</v>
       </c>
       <c r="G23" t="n">
-        <v>10749</v>
+        <v>9672</v>
       </c>
       <c r="H23" t="n">
-        <v>60913</v>
+        <v>54811</v>
       </c>
     </row>
     <row r="24">
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>71662</v>
+        <v>66137</v>
       </c>
       <c r="G24" t="n">
-        <v>10749</v>
+        <v>9920</v>
       </c>
       <c r="H24" t="n">
-        <v>60913</v>
+        <v>56217</v>
       </c>
     </row>
     <row r="25">
@@ -1313,13 +1313,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>71662</v>
+        <v>81840</v>
       </c>
       <c r="G25" t="n">
-        <v>10749</v>
+        <v>12276</v>
       </c>
       <c r="H25" t="n">
-        <v>60913</v>
+        <v>69564</v>
       </c>
     </row>
     <row r="26">
@@ -1349,13 +1349,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>71662</v>
+        <v>65029</v>
       </c>
       <c r="G26" t="n">
-        <v>10749</v>
+        <v>9754</v>
       </c>
       <c r="H26" t="n">
-        <v>60913</v>
+        <v>55275</v>
       </c>
     </row>
     <row r="27">
@@ -1385,13 +1385,13 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>71662</v>
+        <v>82960</v>
       </c>
       <c r="G27" t="n">
-        <v>10749</v>
+        <v>12444</v>
       </c>
       <c r="H27" t="n">
-        <v>60913</v>
+        <v>70516</v>
       </c>
     </row>
     <row r="28">
@@ -1421,13 +1421,13 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>71662</v>
+        <v>66189</v>
       </c>
       <c r="G28" t="n">
-        <v>10749</v>
+        <v>9928</v>
       </c>
       <c r="H28" t="n">
-        <v>60913</v>
+        <v>56261</v>
       </c>
     </row>
     <row r="29">
@@ -1448,22 +1448,22 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2021-08-01</t>
+          <t>2021-09-01</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Aug 2021</t>
+          <t>Sep 2021</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>71662</v>
+        <v>83186</v>
       </c>
       <c r="G29" t="n">
-        <v>10749</v>
+        <v>12477</v>
       </c>
       <c r="H29" t="n">
-        <v>60913</v>
+        <v>70709</v>
       </c>
     </row>
     <row r="30">
@@ -1484,22 +1484,22 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2021-09-01</t>
+          <t>2021-10-01</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Sep 2021</t>
+          <t>Oct 2021</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>71662</v>
+        <v>64009</v>
       </c>
       <c r="G30" t="n">
-        <v>10749</v>
+        <v>9601</v>
       </c>
       <c r="H30" t="n">
-        <v>60913</v>
+        <v>54408</v>
       </c>
     </row>
     <row r="31">
@@ -1520,22 +1520,22 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2021-10-01</t>
+          <t>2022-01-01</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Oct 2021</t>
+          <t>Jan 2022</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>71662</v>
+        <v>64152</v>
       </c>
       <c r="G31" t="n">
-        <v>10749</v>
+        <v>9622</v>
       </c>
       <c r="H31" t="n">
-        <v>60913</v>
+        <v>54530</v>
       </c>
     </row>
     <row r="32">
@@ -1556,22 +1556,22 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2021-12-01</t>
+          <t>2022-02-01</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Dec 2021</t>
+          <t>Feb 2022</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>71662</v>
+        <v>65883</v>
       </c>
       <c r="G32" t="n">
-        <v>10749</v>
+        <v>9882</v>
       </c>
       <c r="H32" t="n">
-        <v>60913</v>
+        <v>56001</v>
       </c>
     </row>
     <row r="33">
@@ -1592,22 +1592,22 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2022-01-01</t>
+          <t>2022-03-01</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Jan 2022</t>
+          <t>Mar 2022</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>75245</v>
+        <v>75297</v>
       </c>
       <c r="G33" t="n">
-        <v>11286</v>
+        <v>11294</v>
       </c>
       <c r="H33" t="n">
-        <v>63959</v>
+        <v>64003</v>
       </c>
     </row>
     <row r="34">
@@ -1628,22 +1628,22 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2022-03-01</t>
+          <t>2022-04-01</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Mar 2022</t>
+          <t>Apr 2022</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>75245</v>
+        <v>63804</v>
       </c>
       <c r="G34" t="n">
-        <v>11286</v>
+        <v>9570</v>
       </c>
       <c r="H34" t="n">
-        <v>63959</v>
+        <v>54234</v>
       </c>
     </row>
     <row r="35">
@@ -1664,22 +1664,22 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2022-04-01</t>
+          <t>2022-05-01</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Apr 2022</t>
+          <t>May 2022</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>75245</v>
+        <v>64054</v>
       </c>
       <c r="G35" t="n">
-        <v>11286</v>
+        <v>9608</v>
       </c>
       <c r="H35" t="n">
-        <v>63959</v>
+        <v>54446</v>
       </c>
     </row>
     <row r="36">
@@ -1709,13 +1709,13 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>75245</v>
+        <v>77664</v>
       </c>
       <c r="G36" t="n">
-        <v>11286</v>
+        <v>11649</v>
       </c>
       <c r="H36" t="n">
-        <v>63959</v>
+        <v>66015</v>
       </c>
     </row>
     <row r="37">
@@ -1736,22 +1736,22 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2022-08-01</t>
+          <t>2022-07-01</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Aug 2022</t>
+          <t>Jul 2022</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>75245</v>
+        <v>64676</v>
       </c>
       <c r="G37" t="n">
-        <v>11286</v>
+        <v>9701</v>
       </c>
       <c r="H37" t="n">
-        <v>63959</v>
+        <v>54975</v>
       </c>
     </row>
     <row r="38">
@@ -1772,22 +1772,22 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2022-09-01</t>
+          <t>2022-08-01</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Sep 2022</t>
+          <t>Aug 2022</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>75245</v>
+        <v>64584</v>
       </c>
       <c r="G38" t="n">
-        <v>11286</v>
+        <v>9687</v>
       </c>
       <c r="H38" t="n">
-        <v>63959</v>
+        <v>54897</v>
       </c>
     </row>
     <row r="39">
@@ -1808,22 +1808,22 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>2022-10-01</t>
+          <t>2022-09-01</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Oct 2022</t>
+          <t>Sep 2022</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>75245</v>
+        <v>79531</v>
       </c>
       <c r="G39" t="n">
-        <v>11286</v>
+        <v>11929</v>
       </c>
       <c r="H39" t="n">
-        <v>63959</v>
+        <v>67602</v>
       </c>
     </row>
     <row r="40">
@@ -1844,22 +1844,22 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2022-11-01</t>
+          <t>2022-10-01</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Nov 2022</t>
+          <t>Oct 2022</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>75245</v>
+        <v>64111</v>
       </c>
       <c r="G40" t="n">
-        <v>11286</v>
+        <v>9616</v>
       </c>
       <c r="H40" t="n">
-        <v>63959</v>
+        <v>54495</v>
       </c>
     </row>
     <row r="41">
@@ -1880,22 +1880,22 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>2022-12-01</t>
+          <t>2022-11-01</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Dec 2022</t>
+          <t>Nov 2022</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>75245</v>
+        <v>66074</v>
       </c>
       <c r="G41" t="n">
-        <v>11286</v>
+        <v>9911</v>
       </c>
       <c r="H41" t="n">
-        <v>63959</v>
+        <v>56163</v>
       </c>
     </row>
     <row r="42">
@@ -1916,22 +1916,22 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>2023-01-01</t>
+          <t>2022-12-01</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Jan 2023</t>
+          <t>Dec 2022</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>79007</v>
+        <v>107483</v>
       </c>
       <c r="G42" t="n">
-        <v>11851</v>
+        <v>16122</v>
       </c>
       <c r="H42" t="n">
-        <v>67156</v>
+        <v>91361</v>
       </c>
     </row>
     <row r="43">
@@ -1952,22 +1952,22 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>2023-02-01</t>
+          <t>2023-03-01</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Feb 2023</t>
+          <t>Mar 2023</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>79007</v>
+        <v>79132</v>
       </c>
       <c r="G43" t="n">
-        <v>11851</v>
+        <v>11869</v>
       </c>
       <c r="H43" t="n">
-        <v>67156</v>
+        <v>67263</v>
       </c>
     </row>
     <row r="44">
@@ -1988,22 +1988,22 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>2023-03-01</t>
+          <t>2023-04-01</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Mar 2023</t>
+          <t>Apr 2023</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>79007</v>
+        <v>64095</v>
       </c>
       <c r="G44" t="n">
-        <v>11851</v>
+        <v>9614</v>
       </c>
       <c r="H44" t="n">
-        <v>67156</v>
+        <v>54481</v>
       </c>
     </row>
     <row r="45">
@@ -2024,22 +2024,22 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>2023-04-01</t>
+          <t>2023-05-01</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Apr 2023</t>
+          <t>May 2023</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>79007</v>
+        <v>65776</v>
       </c>
       <c r="G45" t="n">
-        <v>11851</v>
+        <v>9866</v>
       </c>
       <c r="H45" t="n">
-        <v>67156</v>
+        <v>55910</v>
       </c>
     </row>
     <row r="46">
@@ -2060,22 +2060,22 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>2023-05-01</t>
+          <t>2023-06-01</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>May 2023</t>
+          <t>Jun 2023</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>79007</v>
+        <v>76699</v>
       </c>
       <c r="G46" t="n">
-        <v>11851</v>
+        <v>11504</v>
       </c>
       <c r="H46" t="n">
-        <v>67156</v>
+        <v>65195</v>
       </c>
     </row>
     <row r="47">
@@ -2096,22 +2096,22 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>2023-06-01</t>
+          <t>2023-08-01</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Jun 2023</t>
+          <t>Aug 2023</t>
         </is>
       </c>
       <c r="F47" t="n">
-        <v>79007</v>
+        <v>65410</v>
       </c>
       <c r="G47" t="n">
-        <v>11851</v>
+        <v>9811</v>
       </c>
       <c r="H47" t="n">
-        <v>67156</v>
+        <v>55599</v>
       </c>
     </row>
     <row r="48">
@@ -2132,22 +2132,22 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>2023-07-01</t>
+          <t>2023-09-01</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Jul 2023</t>
+          <t>Sep 2023</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>79007</v>
+        <v>77063</v>
       </c>
       <c r="G48" t="n">
-        <v>11851</v>
+        <v>11559</v>
       </c>
       <c r="H48" t="n">
-        <v>67156</v>
+        <v>65504</v>
       </c>
     </row>
     <row r="49">
@@ -2168,22 +2168,22 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2023-08-01</t>
+          <t>2023-10-01</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Aug 2023</t>
+          <t>Oct 2023</t>
         </is>
       </c>
       <c r="F49" t="n">
-        <v>79007</v>
+        <v>64173</v>
       </c>
       <c r="G49" t="n">
-        <v>11851</v>
+        <v>9625</v>
       </c>
       <c r="H49" t="n">
-        <v>67156</v>
+        <v>54548</v>
       </c>
     </row>
     <row r="50">
@@ -2204,22 +2204,22 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>2023-09-01</t>
+          <t>2023-11-01</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Sep 2023</t>
+          <t>Nov 2023</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>79007</v>
+        <v>65112</v>
       </c>
       <c r="G50" t="n">
-        <v>11851</v>
+        <v>9766</v>
       </c>
       <c r="H50" t="n">
-        <v>67156</v>
+        <v>55346</v>
       </c>
     </row>
     <row r="51">
@@ -2249,13 +2249,13 @@
         </is>
       </c>
       <c r="F51" t="n">
-        <v>79007</v>
+        <v>109990</v>
       </c>
       <c r="G51" t="n">
-        <v>11851</v>
+        <v>16498</v>
       </c>
       <c r="H51" t="n">
-        <v>67156</v>
+        <v>93492</v>
       </c>
     </row>
     <row r="52">
@@ -2276,22 +2276,22 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>2019-01-01</t>
+          <t>2019-03-01</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Jan 2019</t>
+          <t>Mar 2019</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>85000</v>
+        <v>102077</v>
       </c>
       <c r="G52" t="n">
-        <v>12750</v>
+        <v>15311</v>
       </c>
       <c r="H52" t="n">
-        <v>72250</v>
+        <v>86766</v>
       </c>
     </row>
     <row r="53">
@@ -2312,22 +2312,22 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>2019-02-01</t>
+          <t>2019-06-01</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Feb 2019</t>
+          <t>Jun 2019</t>
         </is>
       </c>
       <c r="F53" t="n">
-        <v>85000</v>
+        <v>99411</v>
       </c>
       <c r="G53" t="n">
-        <v>12750</v>
+        <v>14911</v>
       </c>
       <c r="H53" t="n">
-        <v>72250</v>
+        <v>84500</v>
       </c>
     </row>
     <row r="54">
@@ -2348,22 +2348,22 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>2019-05-01</t>
+          <t>2019-07-01</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>May 2019</t>
+          <t>Jul 2019</t>
         </is>
       </c>
       <c r="F54" t="n">
-        <v>85000</v>
+        <v>84868</v>
       </c>
       <c r="G54" t="n">
-        <v>12750</v>
+        <v>12730</v>
       </c>
       <c r="H54" t="n">
-        <v>72250</v>
+        <v>72138</v>
       </c>
     </row>
     <row r="55">
@@ -2384,22 +2384,22 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>2019-06-01</t>
+          <t>2019-08-01</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Jun 2019</t>
+          <t>Aug 2019</t>
         </is>
       </c>
       <c r="F55" t="n">
-        <v>85000</v>
+        <v>84065</v>
       </c>
       <c r="G55" t="n">
-        <v>12750</v>
+        <v>12609</v>
       </c>
       <c r="H55" t="n">
-        <v>72250</v>
+        <v>71456</v>
       </c>
     </row>
     <row r="56">
@@ -2420,22 +2420,22 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>2019-07-01</t>
+          <t>2019-09-01</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Jul 2019</t>
+          <t>Sep 2019</t>
         </is>
       </c>
       <c r="F56" t="n">
-        <v>85000</v>
+        <v>99964</v>
       </c>
       <c r="G56" t="n">
-        <v>12750</v>
+        <v>14994</v>
       </c>
       <c r="H56" t="n">
-        <v>72250</v>
+        <v>84970</v>
       </c>
     </row>
     <row r="57">
@@ -2456,22 +2456,22 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>2019-08-01</t>
+          <t>2019-10-01</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Aug 2019</t>
+          <t>Oct 2019</t>
         </is>
       </c>
       <c r="F57" t="n">
-        <v>85000</v>
+        <v>85003</v>
       </c>
       <c r="G57" t="n">
         <v>12750</v>
       </c>
       <c r="H57" t="n">
-        <v>72250</v>
+        <v>72253</v>
       </c>
     </row>
     <row r="58">
@@ -2492,22 +2492,22 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>2019-09-01</t>
+          <t>2019-11-01</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Sep 2019</t>
+          <t>Nov 2019</t>
         </is>
       </c>
       <c r="F58" t="n">
-        <v>85000</v>
+        <v>85025</v>
       </c>
       <c r="G58" t="n">
-        <v>12750</v>
+        <v>12753</v>
       </c>
       <c r="H58" t="n">
-        <v>72250</v>
+        <v>72272</v>
       </c>
     </row>
     <row r="59">
@@ -2528,22 +2528,22 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>2019-10-01</t>
+          <t>2019-12-01</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Oct 2019</t>
+          <t>Dec 2019</t>
         </is>
       </c>
       <c r="F59" t="n">
-        <v>85000</v>
+        <v>162201</v>
       </c>
       <c r="G59" t="n">
-        <v>12750</v>
+        <v>24330</v>
       </c>
       <c r="H59" t="n">
-        <v>72250</v>
+        <v>137871</v>
       </c>
     </row>
     <row r="60">
@@ -2564,22 +2564,22 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>2019-12-01</t>
+          <t>2020-01-01</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Dec 2019</t>
+          <t>Jan 2020</t>
         </is>
       </c>
       <c r="F60" t="n">
-        <v>85000</v>
+        <v>84266</v>
       </c>
       <c r="G60" t="n">
-        <v>12750</v>
+        <v>12639</v>
       </c>
       <c r="H60" t="n">
-        <v>72250</v>
+        <v>71627</v>
       </c>
     </row>
     <row r="61">
@@ -2600,22 +2600,22 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>2020-02-01</t>
+          <t>2020-03-01</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Feb 2020</t>
+          <t>Mar 2020</t>
         </is>
       </c>
       <c r="F61" t="n">
-        <v>89250</v>
+        <v>103284</v>
       </c>
       <c r="G61" t="n">
-        <v>13387</v>
+        <v>15492</v>
       </c>
       <c r="H61" t="n">
-        <v>75863</v>
+        <v>87792</v>
       </c>
     </row>
     <row r="62">
@@ -2636,22 +2636,22 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>2020-03-01</t>
+          <t>2020-04-01</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Mar 2020</t>
+          <t>Apr 2020</t>
         </is>
       </c>
       <c r="F62" t="n">
-        <v>89250</v>
+        <v>83522</v>
       </c>
       <c r="G62" t="n">
-        <v>13387</v>
+        <v>12528</v>
       </c>
       <c r="H62" t="n">
-        <v>75863</v>
+        <v>70994</v>
       </c>
     </row>
     <row r="63">
@@ -2672,22 +2672,22 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>2020-04-01</t>
+          <t>2020-05-01</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Apr 2020</t>
+          <t>May 2020</t>
         </is>
       </c>
       <c r="F63" t="n">
-        <v>89250</v>
+        <v>83684</v>
       </c>
       <c r="G63" t="n">
-        <v>13387</v>
+        <v>12552</v>
       </c>
       <c r="H63" t="n">
-        <v>75863</v>
+        <v>71132</v>
       </c>
     </row>
     <row r="64">
@@ -2708,22 +2708,22 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>2020-05-01</t>
+          <t>2020-06-01</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>May 2020</t>
+          <t>Jun 2020</t>
         </is>
       </c>
       <c r="F64" t="n">
-        <v>89250</v>
+        <v>96427</v>
       </c>
       <c r="G64" t="n">
-        <v>13387</v>
+        <v>14464</v>
       </c>
       <c r="H64" t="n">
-        <v>75863</v>
+        <v>81963</v>
       </c>
     </row>
     <row r="65">
@@ -2744,22 +2744,22 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>2020-06-01</t>
+          <t>2020-07-01</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Jun 2020</t>
+          <t>Jul 2020</t>
         </is>
       </c>
       <c r="F65" t="n">
-        <v>89250</v>
+        <v>84811</v>
       </c>
       <c r="G65" t="n">
-        <v>13387</v>
+        <v>12721</v>
       </c>
       <c r="H65" t="n">
-        <v>75863</v>
+        <v>72090</v>
       </c>
     </row>
     <row r="66">
@@ -2780,22 +2780,22 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>2020-07-01</t>
+          <t>2020-08-01</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Jul 2020</t>
+          <t>Aug 2020</t>
         </is>
       </c>
       <c r="F66" t="n">
-        <v>89250</v>
+        <v>85506</v>
       </c>
       <c r="G66" t="n">
-        <v>13387</v>
+        <v>12825</v>
       </c>
       <c r="H66" t="n">
-        <v>75863</v>
+        <v>72681</v>
       </c>
     </row>
     <row r="67">
@@ -2816,22 +2816,22 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>2020-08-01</t>
+          <t>2020-10-01</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Aug 2020</t>
+          <t>Oct 2020</t>
         </is>
       </c>
       <c r="F67" t="n">
-        <v>89250</v>
+        <v>84437</v>
       </c>
       <c r="G67" t="n">
-        <v>13387</v>
+        <v>12665</v>
       </c>
       <c r="H67" t="n">
-        <v>75863</v>
+        <v>71772</v>
       </c>
     </row>
     <row r="68">
@@ -2852,22 +2852,22 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>2020-09-01</t>
+          <t>2020-11-01</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Sep 2020</t>
+          <t>Nov 2020</t>
         </is>
       </c>
       <c r="F68" t="n">
-        <v>89250</v>
+        <v>84429</v>
       </c>
       <c r="G68" t="n">
-        <v>13387</v>
+        <v>12664</v>
       </c>
       <c r="H68" t="n">
-        <v>75863</v>
+        <v>71765</v>
       </c>
     </row>
     <row r="69">
@@ -2888,22 +2888,22 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>2020-10-01</t>
+          <t>2020-12-01</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Oct 2020</t>
+          <t>Dec 2020</t>
         </is>
       </c>
       <c r="F69" t="n">
-        <v>89250</v>
+        <v>163293</v>
       </c>
       <c r="G69" t="n">
-        <v>13387</v>
+        <v>24493</v>
       </c>
       <c r="H69" t="n">
-        <v>75863</v>
+        <v>138800</v>
       </c>
     </row>
     <row r="70">
@@ -2924,22 +2924,22 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>2020-12-01</t>
+          <t>2021-01-01</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Dec 2020</t>
+          <t>Jan 2021</t>
         </is>
       </c>
       <c r="F70" t="n">
-        <v>89250</v>
+        <v>83681</v>
       </c>
       <c r="G70" t="n">
-        <v>13387</v>
+        <v>12552</v>
       </c>
       <c r="H70" t="n">
-        <v>75863</v>
+        <v>71129</v>
       </c>
     </row>
     <row r="71">
@@ -2960,22 +2960,22 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>2021-01-01</t>
+          <t>2021-02-01</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Jan 2021</t>
+          <t>Feb 2021</t>
         </is>
       </c>
       <c r="F71" t="n">
-        <v>93712</v>
+        <v>85852</v>
       </c>
       <c r="G71" t="n">
-        <v>14056</v>
+        <v>12877</v>
       </c>
       <c r="H71" t="n">
-        <v>79656</v>
+        <v>72975</v>
       </c>
     </row>
     <row r="72">
@@ -2996,22 +2996,22 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>2021-02-01</t>
+          <t>2021-03-01</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Feb 2021</t>
+          <t>Mar 2021</t>
         </is>
       </c>
       <c r="F72" t="n">
-        <v>93712</v>
+        <v>105472</v>
       </c>
       <c r="G72" t="n">
-        <v>14056</v>
+        <v>15820</v>
       </c>
       <c r="H72" t="n">
-        <v>79656</v>
+        <v>89652</v>
       </c>
     </row>
     <row r="73">
@@ -3032,22 +3032,22 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>2021-03-01</t>
+          <t>2021-04-01</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Mar 2021</t>
+          <t>Apr 2021</t>
         </is>
       </c>
       <c r="F73" t="n">
-        <v>93712</v>
+        <v>85195</v>
       </c>
       <c r="G73" t="n">
-        <v>14056</v>
+        <v>12779</v>
       </c>
       <c r="H73" t="n">
-        <v>79656</v>
+        <v>72416</v>
       </c>
     </row>
     <row r="74">
@@ -3068,22 +3068,22 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>2021-04-01</t>
+          <t>2021-05-01</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Apr 2021</t>
+          <t>May 2021</t>
         </is>
       </c>
       <c r="F74" t="n">
-        <v>93712</v>
+        <v>84959</v>
       </c>
       <c r="G74" t="n">
-        <v>14056</v>
+        <v>12743</v>
       </c>
       <c r="H74" t="n">
-        <v>79656</v>
+        <v>72216</v>
       </c>
     </row>
     <row r="75">
@@ -3113,13 +3113,13 @@
         </is>
       </c>
       <c r="F75" t="n">
-        <v>93712</v>
+        <v>98979</v>
       </c>
       <c r="G75" t="n">
-        <v>14056</v>
+        <v>14846</v>
       </c>
       <c r="H75" t="n">
-        <v>79656</v>
+        <v>84133</v>
       </c>
     </row>
     <row r="76">
@@ -3149,13 +3149,13 @@
         </is>
       </c>
       <c r="F76" t="n">
-        <v>93712</v>
+        <v>83903</v>
       </c>
       <c r="G76" t="n">
-        <v>14056</v>
+        <v>12585</v>
       </c>
       <c r="H76" t="n">
-        <v>79656</v>
+        <v>71318</v>
       </c>
     </row>
     <row r="77">
@@ -3185,13 +3185,13 @@
         </is>
       </c>
       <c r="F77" t="n">
-        <v>93712</v>
+        <v>85794</v>
       </c>
       <c r="G77" t="n">
-        <v>14056</v>
+        <v>12869</v>
       </c>
       <c r="H77" t="n">
-        <v>79656</v>
+        <v>72925</v>
       </c>
     </row>
     <row r="78">
@@ -3221,13 +3221,13 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>93712</v>
+        <v>107914</v>
       </c>
       <c r="G78" t="n">
-        <v>14056</v>
+        <v>16187</v>
       </c>
       <c r="H78" t="n">
-        <v>79656</v>
+        <v>91727</v>
       </c>
     </row>
     <row r="79">
@@ -3257,13 +3257,13 @@
         </is>
       </c>
       <c r="F79" t="n">
-        <v>93712</v>
+        <v>84569</v>
       </c>
       <c r="G79" t="n">
-        <v>14056</v>
+        <v>12685</v>
       </c>
       <c r="H79" t="n">
-        <v>79656</v>
+        <v>71884</v>
       </c>
     </row>
     <row r="80">
@@ -3293,13 +3293,13 @@
         </is>
       </c>
       <c r="F80" t="n">
-        <v>93712</v>
+        <v>85778</v>
       </c>
       <c r="G80" t="n">
-        <v>14056</v>
+        <v>12866</v>
       </c>
       <c r="H80" t="n">
-        <v>79656</v>
+        <v>72912</v>
       </c>
     </row>
     <row r="81">
@@ -3329,13 +3329,13 @@
         </is>
       </c>
       <c r="F81" t="n">
-        <v>93712</v>
+        <v>157603</v>
       </c>
       <c r="G81" t="n">
-        <v>14056</v>
+        <v>23640</v>
       </c>
       <c r="H81" t="n">
-        <v>79656</v>
+        <v>133963</v>
       </c>
     </row>
     <row r="82">
@@ -3365,13 +3365,13 @@
         </is>
       </c>
       <c r="F82" t="n">
-        <v>98397</v>
+        <v>84273</v>
       </c>
       <c r="G82" t="n">
-        <v>14759</v>
+        <v>12640</v>
       </c>
       <c r="H82" t="n">
-        <v>83638</v>
+        <v>71633</v>
       </c>
     </row>
     <row r="83">
@@ -3401,13 +3401,13 @@
         </is>
       </c>
       <c r="F83" t="n">
-        <v>98397</v>
+        <v>84827</v>
       </c>
       <c r="G83" t="n">
-        <v>14759</v>
+        <v>12724</v>
       </c>
       <c r="H83" t="n">
-        <v>83638</v>
+        <v>72103</v>
       </c>
     </row>
     <row r="84">
@@ -3437,13 +3437,13 @@
         </is>
       </c>
       <c r="F84" t="n">
-        <v>98397</v>
+        <v>103709</v>
       </c>
       <c r="G84" t="n">
-        <v>14759</v>
+        <v>15556</v>
       </c>
       <c r="H84" t="n">
-        <v>83638</v>
+        <v>88153</v>
       </c>
     </row>
     <row r="85">
@@ -3473,13 +3473,13 @@
         </is>
       </c>
       <c r="F85" t="n">
-        <v>98397</v>
+        <v>86328</v>
       </c>
       <c r="G85" t="n">
-        <v>14759</v>
+        <v>12949</v>
       </c>
       <c r="H85" t="n">
-        <v>83638</v>
+        <v>73379</v>
       </c>
     </row>
     <row r="86">
@@ -3500,22 +3500,22 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>2022-06-01</t>
+          <t>2022-05-01</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Jun 2022</t>
+          <t>May 2022</t>
         </is>
       </c>
       <c r="F86" t="n">
-        <v>98397</v>
+        <v>86144</v>
       </c>
       <c r="G86" t="n">
-        <v>14759</v>
+        <v>12921</v>
       </c>
       <c r="H86" t="n">
-        <v>83638</v>
+        <v>73223</v>
       </c>
     </row>
     <row r="87">
@@ -3536,22 +3536,22 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>2022-07-01</t>
+          <t>2022-06-01</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Jul 2022</t>
+          <t>Jun 2022</t>
         </is>
       </c>
       <c r="F87" t="n">
-        <v>98397</v>
+        <v>99902</v>
       </c>
       <c r="G87" t="n">
-        <v>14759</v>
+        <v>14985</v>
       </c>
       <c r="H87" t="n">
-        <v>83638</v>
+        <v>84917</v>
       </c>
     </row>
     <row r="88">
@@ -3572,22 +3572,22 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>2022-08-01</t>
+          <t>2022-07-01</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Aug 2022</t>
+          <t>Jul 2022</t>
         </is>
       </c>
       <c r="F88" t="n">
-        <v>98397</v>
+        <v>85865</v>
       </c>
       <c r="G88" t="n">
-        <v>14759</v>
+        <v>12879</v>
       </c>
       <c r="H88" t="n">
-        <v>83638</v>
+        <v>72986</v>
       </c>
     </row>
     <row r="89">
@@ -3608,22 +3608,22 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>2022-09-01</t>
+          <t>2022-08-01</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Sep 2022</t>
+          <t>Aug 2022</t>
         </is>
       </c>
       <c r="F89" t="n">
-        <v>98397</v>
+        <v>83773</v>
       </c>
       <c r="G89" t="n">
-        <v>14759</v>
+        <v>12565</v>
       </c>
       <c r="H89" t="n">
-        <v>83638</v>
+        <v>71208</v>
       </c>
     </row>
     <row r="90">
@@ -3644,22 +3644,22 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>2022-10-01</t>
+          <t>2022-09-01</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Oct 2022</t>
+          <t>Sep 2022</t>
         </is>
       </c>
       <c r="F90" t="n">
-        <v>98397</v>
+        <v>96407</v>
       </c>
       <c r="G90" t="n">
-        <v>14759</v>
+        <v>14461</v>
       </c>
       <c r="H90" t="n">
-        <v>83638</v>
+        <v>81946</v>
       </c>
     </row>
     <row r="91">
@@ -3689,13 +3689,13 @@
         </is>
       </c>
       <c r="F91" t="n">
-        <v>98397</v>
+        <v>85820</v>
       </c>
       <c r="G91" t="n">
-        <v>14759</v>
+        <v>12873</v>
       </c>
       <c r="H91" t="n">
-        <v>83638</v>
+        <v>72947</v>
       </c>
     </row>
     <row r="92">
@@ -3725,13 +3725,13 @@
         </is>
       </c>
       <c r="F92" t="n">
-        <v>98397</v>
+        <v>164038</v>
       </c>
       <c r="G92" t="n">
-        <v>14759</v>
+        <v>24605</v>
       </c>
       <c r="H92" t="n">
-        <v>83638</v>
+        <v>139433</v>
       </c>
     </row>
     <row r="93">
@@ -3752,22 +3752,22 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>2023-02-01</t>
+          <t>2023-01-01</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Feb 2023</t>
+          <t>Jan 2023</t>
         </is>
       </c>
       <c r="F93" t="n">
-        <v>103316</v>
+        <v>85500</v>
       </c>
       <c r="G93" t="n">
-        <v>15497</v>
+        <v>12825</v>
       </c>
       <c r="H93" t="n">
-        <v>87819</v>
+        <v>72675</v>
       </c>
     </row>
     <row r="94">
@@ -3788,22 +3788,22 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>2023-04-01</t>
+          <t>2023-02-01</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Apr 2023</t>
+          <t>Feb 2023</t>
         </is>
       </c>
       <c r="F94" t="n">
-        <v>103316</v>
+        <v>84609</v>
       </c>
       <c r="G94" t="n">
-        <v>15497</v>
+        <v>12691</v>
       </c>
       <c r="H94" t="n">
-        <v>87819</v>
+        <v>71918</v>
       </c>
     </row>
     <row r="95">
@@ -3824,22 +3824,22 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>2023-05-01</t>
+          <t>2023-04-01</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>May 2023</t>
+          <t>Apr 2023</t>
         </is>
       </c>
       <c r="F95" t="n">
-        <v>103316</v>
+        <v>85447</v>
       </c>
       <c r="G95" t="n">
-        <v>15497</v>
+        <v>12817</v>
       </c>
       <c r="H95" t="n">
-        <v>87819</v>
+        <v>72630</v>
       </c>
     </row>
     <row r="96">
@@ -3860,22 +3860,22 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>2023-06-01</t>
+          <t>2023-05-01</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Jun 2023</t>
+          <t>May 2023</t>
         </is>
       </c>
       <c r="F96" t="n">
-        <v>103316</v>
+        <v>84775</v>
       </c>
       <c r="G96" t="n">
-        <v>15497</v>
+        <v>12716</v>
       </c>
       <c r="H96" t="n">
-        <v>87819</v>
+        <v>72059</v>
       </c>
     </row>
     <row r="97">
@@ -3896,22 +3896,22 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>2023-07-01</t>
+          <t>2023-06-01</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Jul 2023</t>
+          <t>Jun 2023</t>
         </is>
       </c>
       <c r="F97" t="n">
-        <v>103316</v>
+        <v>100323</v>
       </c>
       <c r="G97" t="n">
-        <v>15497</v>
+        <v>15048</v>
       </c>
       <c r="H97" t="n">
-        <v>87819</v>
+        <v>85275</v>
       </c>
     </row>
     <row r="98">
@@ -3932,22 +3932,22 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>2023-09-01</t>
+          <t>2023-07-01</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Sep 2023</t>
+          <t>Jul 2023</t>
         </is>
       </c>
       <c r="F98" t="n">
-        <v>103316</v>
+        <v>86398</v>
       </c>
       <c r="G98" t="n">
-        <v>15497</v>
+        <v>12959</v>
       </c>
       <c r="H98" t="n">
-        <v>87819</v>
+        <v>73439</v>
       </c>
     </row>
     <row r="99">
@@ -3968,22 +3968,22 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>2023-10-01</t>
+          <t>2023-08-01</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Oct 2023</t>
+          <t>Aug 2023</t>
         </is>
       </c>
       <c r="F99" t="n">
-        <v>103316</v>
+        <v>85119</v>
       </c>
       <c r="G99" t="n">
-        <v>15497</v>
+        <v>12767</v>
       </c>
       <c r="H99" t="n">
-        <v>87819</v>
+        <v>72352</v>
       </c>
     </row>
     <row r="100">
@@ -4004,22 +4004,22 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>2023-11-01</t>
+          <t>2023-10-01</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Nov 2023</t>
+          <t>Oct 2023</t>
         </is>
       </c>
       <c r="F100" t="n">
-        <v>103316</v>
+        <v>84591</v>
       </c>
       <c r="G100" t="n">
-        <v>15497</v>
+        <v>12688</v>
       </c>
       <c r="H100" t="n">
-        <v>87819</v>
+        <v>71903</v>
       </c>
     </row>
     <row r="101">
@@ -4040,22 +4040,22 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>2023-12-01</t>
+          <t>2023-11-01</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Dec 2023</t>
+          <t>Nov 2023</t>
         </is>
       </c>
       <c r="F101" t="n">
-        <v>103316</v>
+        <v>84065</v>
       </c>
       <c r="G101" t="n">
-        <v>15497</v>
+        <v>12609</v>
       </c>
       <c r="H101" t="n">
-        <v>87819</v>
+        <v>71456</v>
       </c>
     </row>
     <row r="102">
@@ -4076,22 +4076,22 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>2019-03-01</t>
+          <t>2019-01-01</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Mar 2019</t>
+          <t>Jan 2019</t>
         </is>
       </c>
       <c r="F102" t="n">
-        <v>50000</v>
+        <v>50083</v>
       </c>
       <c r="G102" t="n">
-        <v>7500</v>
+        <v>7512</v>
       </c>
       <c r="H102" t="n">
-        <v>42500</v>
+        <v>42571</v>
       </c>
     </row>
     <row r="103">
@@ -4112,22 +4112,22 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>2019-04-01</t>
+          <t>2019-02-01</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Apr 2019</t>
+          <t>Feb 2019</t>
         </is>
       </c>
       <c r="F103" t="n">
-        <v>50000</v>
+        <v>50996</v>
       </c>
       <c r="G103" t="n">
-        <v>7500</v>
+        <v>7649</v>
       </c>
       <c r="H103" t="n">
-        <v>42500</v>
+        <v>43347</v>
       </c>
     </row>
     <row r="104">
@@ -4148,22 +4148,22 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>2019-05-01</t>
+          <t>2019-03-01</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>May 2019</t>
+          <t>Mar 2019</t>
         </is>
       </c>
       <c r="F104" t="n">
-        <v>50000</v>
+        <v>64350</v>
       </c>
       <c r="G104" t="n">
-        <v>7500</v>
+        <v>9652</v>
       </c>
       <c r="H104" t="n">
-        <v>42500</v>
+        <v>54698</v>
       </c>
     </row>
     <row r="105">
@@ -4184,22 +4184,22 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>2019-06-01</t>
+          <t>2019-04-01</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Jun 2019</t>
+          <t>Apr 2019</t>
         </is>
       </c>
       <c r="F105" t="n">
-        <v>50000</v>
+        <v>49522</v>
       </c>
       <c r="G105" t="n">
-        <v>7500</v>
+        <v>7428</v>
       </c>
       <c r="H105" t="n">
-        <v>42500</v>
+        <v>42094</v>
       </c>
     </row>
     <row r="106">
@@ -4220,22 +4220,22 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>2019-09-01</t>
+          <t>2019-05-01</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Sep 2019</t>
+          <t>May 2019</t>
         </is>
       </c>
       <c r="F106" t="n">
-        <v>50000</v>
+        <v>50087</v>
       </c>
       <c r="G106" t="n">
-        <v>7500</v>
+        <v>7513</v>
       </c>
       <c r="H106" t="n">
-        <v>42500</v>
+        <v>42574</v>
       </c>
     </row>
     <row r="107">
@@ -4256,22 +4256,22 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>2019-10-01</t>
+          <t>2019-06-01</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Oct 2019</t>
+          <t>Jun 2019</t>
         </is>
       </c>
       <c r="F107" t="n">
-        <v>50000</v>
+        <v>64569</v>
       </c>
       <c r="G107" t="n">
-        <v>7500</v>
+        <v>9685</v>
       </c>
       <c r="H107" t="n">
-        <v>42500</v>
+        <v>54884</v>
       </c>
     </row>
     <row r="108">
@@ -4292,22 +4292,22 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>2019-11-01</t>
+          <t>2019-07-01</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Nov 2019</t>
+          <t>Jul 2019</t>
         </is>
       </c>
       <c r="F108" t="n">
-        <v>50000</v>
+        <v>50843</v>
       </c>
       <c r="G108" t="n">
-        <v>7500</v>
+        <v>7626</v>
       </c>
       <c r="H108" t="n">
-        <v>42500</v>
+        <v>43217</v>
       </c>
     </row>
     <row r="109">
@@ -4328,22 +4328,22 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>2019-12-01</t>
+          <t>2019-08-01</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Dec 2019</t>
+          <t>Aug 2019</t>
         </is>
       </c>
       <c r="F109" t="n">
-        <v>50000</v>
+        <v>50581</v>
       </c>
       <c r="G109" t="n">
-        <v>7500</v>
+        <v>7587</v>
       </c>
       <c r="H109" t="n">
-        <v>42500</v>
+        <v>42994</v>
       </c>
     </row>
     <row r="110">
@@ -4364,22 +4364,22 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>2020-01-01</t>
+          <t>2019-11-01</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Jan 2020</t>
+          <t>Nov 2019</t>
         </is>
       </c>
       <c r="F110" t="n">
-        <v>52500</v>
+        <v>49640</v>
       </c>
       <c r="G110" t="n">
-        <v>7875</v>
+        <v>7446</v>
       </c>
       <c r="H110" t="n">
-        <v>44625</v>
+        <v>42194</v>
       </c>
     </row>
     <row r="111">
@@ -4400,22 +4400,22 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>2020-03-01</t>
+          <t>2020-01-01</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Mar 2020</t>
+          <t>Jan 2020</t>
         </is>
       </c>
       <c r="F111" t="n">
-        <v>60000</v>
+        <v>50026</v>
       </c>
       <c r="G111" t="n">
-        <v>9000</v>
+        <v>7503</v>
       </c>
       <c r="H111" t="n">
-        <v>51000</v>
+        <v>42523</v>
       </c>
     </row>
     <row r="112">
@@ -4436,22 +4436,22 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>2020-04-01</t>
+          <t>2020-02-01</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Apr 2020</t>
+          <t>Feb 2020</t>
         </is>
       </c>
       <c r="F112" t="n">
-        <v>50000</v>
+        <v>49849</v>
       </c>
       <c r="G112" t="n">
-        <v>7500</v>
+        <v>7477</v>
       </c>
       <c r="H112" t="n">
-        <v>42500</v>
+        <v>42372</v>
       </c>
     </row>
     <row r="113">
@@ -4472,22 +4472,22 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>2020-05-01</t>
+          <t>2020-03-01</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>May 2020</t>
+          <t>Mar 2020</t>
         </is>
       </c>
       <c r="F113" t="n">
-        <v>50000</v>
+        <v>61596</v>
       </c>
       <c r="G113" t="n">
-        <v>7500</v>
+        <v>9239</v>
       </c>
       <c r="H113" t="n">
-        <v>42500</v>
+        <v>52357</v>
       </c>
     </row>
     <row r="114">
@@ -4508,22 +4508,22 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>2020-06-01</t>
+          <t>2020-04-01</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Jun 2020</t>
+          <t>Apr 2020</t>
         </is>
       </c>
       <c r="F114" t="n">
-        <v>50000</v>
+        <v>50062</v>
       </c>
       <c r="G114" t="n">
-        <v>7500</v>
+        <v>7509</v>
       </c>
       <c r="H114" t="n">
-        <v>42500</v>
+        <v>42553</v>
       </c>
     </row>
     <row r="115">
@@ -4544,22 +4544,22 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>2020-07-01</t>
+          <t>2020-05-01</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Jul 2020</t>
+          <t>May 2020</t>
         </is>
       </c>
       <c r="F115" t="n">
-        <v>50000</v>
+        <v>49525</v>
       </c>
       <c r="G115" t="n">
-        <v>7500</v>
+        <v>7428</v>
       </c>
       <c r="H115" t="n">
-        <v>42500</v>
+        <v>42097</v>
       </c>
     </row>
     <row r="116">
@@ -4580,22 +4580,22 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>2020-08-01</t>
+          <t>2020-07-01</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Aug 2020</t>
+          <t>Jul 2020</t>
         </is>
       </c>
       <c r="F116" t="n">
-        <v>50000</v>
+        <v>50689</v>
       </c>
       <c r="G116" t="n">
-        <v>7500</v>
+        <v>7603</v>
       </c>
       <c r="H116" t="n">
-        <v>42500</v>
+        <v>43086</v>
       </c>
     </row>
     <row r="117">
@@ -4616,22 +4616,22 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>2020-09-01</t>
+          <t>2020-08-01</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Sep 2020</t>
+          <t>Aug 2020</t>
         </is>
       </c>
       <c r="F117" t="n">
-        <v>50000</v>
+        <v>49791</v>
       </c>
       <c r="G117" t="n">
-        <v>7500</v>
+        <v>7468</v>
       </c>
       <c r="H117" t="n">
-        <v>42500</v>
+        <v>42323</v>
       </c>
     </row>
     <row r="118">
@@ -4661,13 +4661,13 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>50000</v>
+        <v>49601</v>
       </c>
       <c r="G118" t="n">
-        <v>7500</v>
+        <v>7440</v>
       </c>
       <c r="H118" t="n">
-        <v>42500</v>
+        <v>42161</v>
       </c>
     </row>
     <row r="119">
@@ -4697,13 +4697,13 @@
         </is>
       </c>
       <c r="F119" t="n">
-        <v>50000</v>
+        <v>49265</v>
       </c>
       <c r="G119" t="n">
-        <v>7500</v>
+        <v>7389</v>
       </c>
       <c r="H119" t="n">
-        <v>42500</v>
+        <v>41876</v>
       </c>
     </row>
     <row r="120">
@@ -4724,22 +4724,22 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>2020-12-01</t>
+          <t>2021-01-01</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Dec 2020</t>
+          <t>Jan 2021</t>
         </is>
       </c>
       <c r="F120" t="n">
-        <v>50000</v>
+        <v>50914</v>
       </c>
       <c r="G120" t="n">
-        <v>7500</v>
+        <v>7637</v>
       </c>
       <c r="H120" t="n">
-        <v>42500</v>
+        <v>43277</v>
       </c>
     </row>
     <row r="121">
@@ -4760,22 +4760,22 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>2021-01-01</t>
+          <t>2021-02-01</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Jan 2021</t>
+          <t>Feb 2021</t>
         </is>
       </c>
       <c r="F121" t="n">
-        <v>52500</v>
+        <v>50438</v>
       </c>
       <c r="G121" t="n">
-        <v>7875</v>
+        <v>7565</v>
       </c>
       <c r="H121" t="n">
-        <v>44625</v>
+        <v>42873</v>
       </c>
     </row>
     <row r="122">
@@ -4796,22 +4796,22 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>2021-02-01</t>
+          <t>2021-03-01</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Feb 2021</t>
+          <t>Mar 2021</t>
         </is>
       </c>
       <c r="F122" t="n">
-        <v>52500</v>
+        <v>58301</v>
       </c>
       <c r="G122" t="n">
-        <v>7875</v>
+        <v>8745</v>
       </c>
       <c r="H122" t="n">
-        <v>44625</v>
+        <v>49556</v>
       </c>
     </row>
     <row r="123">
@@ -4832,22 +4832,22 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>2021-03-01</t>
+          <t>2021-04-01</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Mar 2021</t>
+          <t>Apr 2021</t>
         </is>
       </c>
       <c r="F123" t="n">
-        <v>52500</v>
+        <v>49114</v>
       </c>
       <c r="G123" t="n">
-        <v>7875</v>
+        <v>7367</v>
       </c>
       <c r="H123" t="n">
-        <v>44625</v>
+        <v>41747</v>
       </c>
     </row>
     <row r="124">
@@ -4868,22 +4868,22 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>2021-04-01</t>
+          <t>2021-05-01</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Apr 2021</t>
+          <t>May 2021</t>
         </is>
       </c>
       <c r="F124" t="n">
-        <v>52500</v>
+        <v>50554</v>
       </c>
       <c r="G124" t="n">
-        <v>7875</v>
+        <v>7583</v>
       </c>
       <c r="H124" t="n">
-        <v>44625</v>
+        <v>42971</v>
       </c>
     </row>
     <row r="125">
@@ -4913,13 +4913,13 @@
         </is>
       </c>
       <c r="F125" t="n">
-        <v>52500</v>
+        <v>58780</v>
       </c>
       <c r="G125" t="n">
-        <v>7875</v>
+        <v>8817</v>
       </c>
       <c r="H125" t="n">
-        <v>44625</v>
+        <v>49963</v>
       </c>
     </row>
     <row r="126">
@@ -4949,13 +4949,13 @@
         </is>
       </c>
       <c r="F126" t="n">
-        <v>52500</v>
+        <v>49381</v>
       </c>
       <c r="G126" t="n">
-        <v>7875</v>
+        <v>7407</v>
       </c>
       <c r="H126" t="n">
-        <v>44625</v>
+        <v>41974</v>
       </c>
     </row>
     <row r="127">
@@ -4976,22 +4976,22 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>2021-10-01</t>
+          <t>2021-09-01</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Oct 2021</t>
+          <t>Sep 2021</t>
         </is>
       </c>
       <c r="F127" t="n">
+        <v>61764</v>
+      </c>
+      <c r="G127" t="n">
+        <v>9264</v>
+      </c>
+      <c r="H127" t="n">
         <v>52500</v>
-      </c>
-      <c r="G127" t="n">
-        <v>7875</v>
-      </c>
-      <c r="H127" t="n">
-        <v>44625</v>
       </c>
     </row>
     <row r="128">
@@ -5012,22 +5012,22 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>2021-11-01</t>
+          <t>2021-10-01</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Nov 2021</t>
+          <t>Oct 2021</t>
         </is>
       </c>
       <c r="F128" t="n">
-        <v>52500</v>
+        <v>49117</v>
       </c>
       <c r="G128" t="n">
-        <v>7875</v>
+        <v>7367</v>
       </c>
       <c r="H128" t="n">
-        <v>44625</v>
+        <v>41750</v>
       </c>
     </row>
     <row r="129">
@@ -5048,22 +5048,22 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>2021-12-01</t>
+          <t>2021-11-01</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Dec 2021</t>
+          <t>Nov 2021</t>
         </is>
       </c>
       <c r="F129" t="n">
-        <v>52500</v>
+        <v>49273</v>
       </c>
       <c r="G129" t="n">
-        <v>7875</v>
+        <v>7390</v>
       </c>
       <c r="H129" t="n">
-        <v>44625</v>
+        <v>41883</v>
       </c>
     </row>
     <row r="130">
@@ -5084,22 +5084,22 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>2022-01-01</t>
+          <t>2021-12-01</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Jan 2022</t>
+          <t>Dec 2021</t>
         </is>
       </c>
       <c r="F130" t="n">
-        <v>55125</v>
+        <v>83907</v>
       </c>
       <c r="G130" t="n">
-        <v>8268</v>
+        <v>12586</v>
       </c>
       <c r="H130" t="n">
-        <v>46857</v>
+        <v>71321</v>
       </c>
     </row>
     <row r="131">
@@ -5120,22 +5120,22 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>2022-02-01</t>
+          <t>2022-01-01</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Feb 2022</t>
+          <t>Jan 2022</t>
         </is>
       </c>
       <c r="F131" t="n">
-        <v>55125</v>
+        <v>50857</v>
       </c>
       <c r="G131" t="n">
-        <v>8268</v>
+        <v>7628</v>
       </c>
       <c r="H131" t="n">
-        <v>46857</v>
+        <v>43229</v>
       </c>
     </row>
     <row r="132">
@@ -5165,13 +5165,13 @@
         </is>
       </c>
       <c r="F132" t="n">
-        <v>55125</v>
+        <v>58813</v>
       </c>
       <c r="G132" t="n">
-        <v>8268</v>
+        <v>8821</v>
       </c>
       <c r="H132" t="n">
-        <v>46857</v>
+        <v>49992</v>
       </c>
     </row>
     <row r="133">
@@ -5201,13 +5201,13 @@
         </is>
       </c>
       <c r="F133" t="n">
-        <v>55125</v>
+        <v>49636</v>
       </c>
       <c r="G133" t="n">
-        <v>8268</v>
+        <v>7445</v>
       </c>
       <c r="H133" t="n">
-        <v>46857</v>
+        <v>42191</v>
       </c>
     </row>
     <row r="134">
@@ -5228,22 +5228,22 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>2022-05-01</t>
+          <t>2022-06-01</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>May 2022</t>
+          <t>Jun 2022</t>
         </is>
       </c>
       <c r="F134" t="n">
-        <v>55125</v>
+        <v>59760</v>
       </c>
       <c r="G134" t="n">
-        <v>8268</v>
+        <v>8964</v>
       </c>
       <c r="H134" t="n">
-        <v>46857</v>
+        <v>50796</v>
       </c>
     </row>
     <row r="135">
@@ -5264,22 +5264,22 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>2022-06-01</t>
+          <t>2022-07-01</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Jun 2022</t>
+          <t>Jul 2022</t>
         </is>
       </c>
       <c r="F135" t="n">
-        <v>55125</v>
+        <v>50142</v>
       </c>
       <c r="G135" t="n">
-        <v>8268</v>
+        <v>7521</v>
       </c>
       <c r="H135" t="n">
-        <v>46857</v>
+        <v>42621</v>
       </c>
     </row>
     <row r="136">
@@ -5300,22 +5300,22 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>2022-07-01</t>
+          <t>2022-08-01</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Jul 2022</t>
+          <t>Aug 2022</t>
         </is>
       </c>
       <c r="F136" t="n">
-        <v>65000</v>
+        <v>49078</v>
       </c>
       <c r="G136" t="n">
-        <v>9750</v>
+        <v>7361</v>
       </c>
       <c r="H136" t="n">
-        <v>55250</v>
+        <v>41717</v>
       </c>
     </row>
     <row r="137">
@@ -5336,22 +5336,22 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>2022-08-01</t>
+          <t>2022-10-01</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Aug 2022</t>
+          <t>Oct 2022</t>
         </is>
       </c>
       <c r="F137" t="n">
-        <v>65000</v>
+        <v>49481</v>
       </c>
       <c r="G137" t="n">
-        <v>9750</v>
+        <v>7422</v>
       </c>
       <c r="H137" t="n">
-        <v>55250</v>
+        <v>42059</v>
       </c>
     </row>
     <row r="138">
@@ -5372,22 +5372,22 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>2022-09-01</t>
+          <t>2022-11-01</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Sep 2022</t>
+          <t>Nov 2022</t>
         </is>
       </c>
       <c r="F138" t="n">
-        <v>55000</v>
+        <v>49585</v>
       </c>
       <c r="G138" t="n">
-        <v>8250</v>
+        <v>7437</v>
       </c>
       <c r="H138" t="n">
-        <v>46750</v>
+        <v>42148</v>
       </c>
     </row>
     <row r="139">
@@ -5408,22 +5408,22 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>2022-10-01</t>
+          <t>2022-12-01</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Oct 2022</t>
+          <t>Dec 2022</t>
         </is>
       </c>
       <c r="F139" t="n">
-        <v>55000</v>
+        <v>82587</v>
       </c>
       <c r="G139" t="n">
-        <v>8250</v>
+        <v>12388</v>
       </c>
       <c r="H139" t="n">
-        <v>46750</v>
+        <v>70199</v>
       </c>
     </row>
     <row r="140">
@@ -5444,22 +5444,22 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>2022-11-01</t>
+          <t>2023-01-01</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Nov 2022</t>
+          <t>Jan 2023</t>
         </is>
       </c>
       <c r="F140" t="n">
-        <v>55000</v>
+        <v>50048</v>
       </c>
       <c r="G140" t="n">
-        <v>8250</v>
+        <v>7507</v>
       </c>
       <c r="H140" t="n">
-        <v>46750</v>
+        <v>42541</v>
       </c>
     </row>
     <row r="141">
@@ -5480,22 +5480,22 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>2023-01-01</t>
+          <t>2023-02-01</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Jan 2023</t>
+          <t>Feb 2023</t>
         </is>
       </c>
       <c r="F141" t="n">
-        <v>57750</v>
+        <v>49322</v>
       </c>
       <c r="G141" t="n">
-        <v>8662</v>
+        <v>7398</v>
       </c>
       <c r="H141" t="n">
-        <v>49088</v>
+        <v>41924</v>
       </c>
     </row>
     <row r="142">
@@ -5516,22 +5516,22 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>2023-02-01</t>
+          <t>2023-03-01</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Feb 2023</t>
+          <t>Mar 2023</t>
         </is>
       </c>
       <c r="F142" t="n">
-        <v>57750</v>
+        <v>64341</v>
       </c>
       <c r="G142" t="n">
-        <v>8662</v>
+        <v>9651</v>
       </c>
       <c r="H142" t="n">
-        <v>49088</v>
+        <v>54690</v>
       </c>
     </row>
     <row r="143">
@@ -5552,22 +5552,22 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>2023-03-01</t>
+          <t>2023-04-01</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Mar 2023</t>
+          <t>Apr 2023</t>
         </is>
       </c>
       <c r="F143" t="n">
-        <v>57750</v>
+        <v>49236</v>
       </c>
       <c r="G143" t="n">
-        <v>8662</v>
+        <v>7385</v>
       </c>
       <c r="H143" t="n">
-        <v>49088</v>
+        <v>41851</v>
       </c>
     </row>
     <row r="144">
@@ -5597,13 +5597,13 @@
         </is>
       </c>
       <c r="F144" t="n">
-        <v>57750</v>
+        <v>50756</v>
       </c>
       <c r="G144" t="n">
-        <v>8662</v>
+        <v>7613</v>
       </c>
       <c r="H144" t="n">
-        <v>49088</v>
+        <v>43143</v>
       </c>
     </row>
     <row r="145">
@@ -5633,13 +5633,13 @@
         </is>
       </c>
       <c r="F145" t="n">
-        <v>57750</v>
+        <v>64798</v>
       </c>
       <c r="G145" t="n">
-        <v>8662</v>
+        <v>9719</v>
       </c>
       <c r="H145" t="n">
-        <v>49088</v>
+        <v>55079</v>
       </c>
     </row>
     <row r="146">
@@ -5669,13 +5669,13 @@
         </is>
       </c>
       <c r="F146" t="n">
-        <v>57750</v>
+        <v>50437</v>
       </c>
       <c r="G146" t="n">
-        <v>8662</v>
+        <v>7565</v>
       </c>
       <c r="H146" t="n">
-        <v>49088</v>
+        <v>42872</v>
       </c>
     </row>
     <row r="147">
@@ -5705,13 +5705,13 @@
         </is>
       </c>
       <c r="F147" t="n">
-        <v>57750</v>
+        <v>50038</v>
       </c>
       <c r="G147" t="n">
-        <v>8662</v>
+        <v>7505</v>
       </c>
       <c r="H147" t="n">
-        <v>49088</v>
+        <v>42533</v>
       </c>
     </row>
     <row r="148">
@@ -5741,13 +5741,13 @@
         </is>
       </c>
       <c r="F148" t="n">
-        <v>57750</v>
+        <v>59895</v>
       </c>
       <c r="G148" t="n">
-        <v>8662</v>
+        <v>8984</v>
       </c>
       <c r="H148" t="n">
-        <v>49088</v>
+        <v>50911</v>
       </c>
     </row>
     <row r="149">
@@ -5777,13 +5777,13 @@
         </is>
       </c>
       <c r="F149" t="n">
-        <v>57750</v>
+        <v>50385</v>
       </c>
       <c r="G149" t="n">
-        <v>8662</v>
+        <v>7557</v>
       </c>
       <c r="H149" t="n">
-        <v>49088</v>
+        <v>42828</v>
       </c>
     </row>
     <row r="150">
@@ -5813,13 +5813,13 @@
         </is>
       </c>
       <c r="F150" t="n">
-        <v>57750</v>
+        <v>49287</v>
       </c>
       <c r="G150" t="n">
-        <v>8662</v>
+        <v>7393</v>
       </c>
       <c r="H150" t="n">
-        <v>49088</v>
+        <v>41894</v>
       </c>
     </row>
     <row r="151">
@@ -5849,13 +5849,13 @@
         </is>
       </c>
       <c r="F151" t="n">
-        <v>57750</v>
+        <v>80995</v>
       </c>
       <c r="G151" t="n">
-        <v>8662</v>
+        <v>12149</v>
       </c>
       <c r="H151" t="n">
-        <v>49088</v>
+        <v>68846</v>
       </c>
     </row>
   </sheetData>

</xml_diff>